<commit_message>
Completely removed gemini from .tex file as well. Now, fixing qwen3.5 model. now replacing it with another qwen model
</commit_message>
<xml_diff>
--- a/progress_chart/final_gnatt_chart.xlsx
+++ b/progress_chart/final_gnatt_chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\OneDrive - Southampton Solent University\COM726 - Dissertation\charts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\OneDrive - Southampton Solent University\COM726 - Dissertation\progress_chart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3828E78B-162D-4A93-9F94-CC16F53F3465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49435718-F8F1-4C43-9B89-D35A80D497A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -381,14 +381,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -796,14 +796,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:1901" ht="23.35" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="3" spans="1:1901" x14ac:dyDescent="0.5">
       <c r="A3" s="18" t="s">
@@ -822,7 +822,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="19">
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="C4" s="18"/>
       <c r="D4" s="18"/>
@@ -835,7 +835,7 @@
       </c>
       <c r="B5" s="19">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46143</v>
       </c>
       <c r="C5" s="18"/>
       <c r="D5" s="18"/>
@@ -848,7 +848,7 @@
       </c>
       <c r="B6" s="18">
         <f ca="1">ROUNDUP((B5-B3)/7,0)</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C6" s="18"/>
       <c r="D6" s="18"/>
@@ -856,7 +856,7 @@
       <c r="F6" s="18"/>
     </row>
     <row r="7" spans="1:1901" x14ac:dyDescent="0.5">
-      <c r="K7" s="34"/>
+      <c r="K7" s="32"/>
     </row>
     <row r="10" spans="1:1901" x14ac:dyDescent="0.5">
       <c r="A10" s="2"/>
@@ -1005,10 +1005,10 @@
       <c r="Y11" s="17"/>
     </row>
     <row r="12" spans="1:1901" s="7" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="33"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -2978,18 +2978,17 @@
         <v>46042</v>
       </c>
       <c r="C15" s="24">
-        <f ca="1">B5</f>
-        <v>46064</v>
+        <v>46085</v>
       </c>
       <c r="D15" s="23">
-        <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <f t="shared" si="1"/>
+        <v>43</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="25">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="G15" s="26"/>
       <c r="H15" s="12"/>
@@ -3018,18 +3017,17 @@
         <v>46042</v>
       </c>
       <c r="C16" s="24">
-        <f ca="1">B5</f>
-        <v>46064</v>
+        <v>46057</v>
       </c>
       <c r="D16" s="23">
-        <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <f t="shared" si="1"/>
+        <v>15</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F16" s="25">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="G16" s="26"/>
       <c r="H16" s="12"/>
@@ -3135,18 +3133,17 @@
         <v>46054</v>
       </c>
       <c r="C19" s="24">
-        <f ca="1">B5</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
       <c r="D19" s="23">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="E19" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="23" t="s">
-        <v>9</v>
-      </c>
       <c r="F19" s="25">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G19" s="26"/>
       <c r="H19" s="12"/>
@@ -3184,7 +3181,7 @@
         <v>10</v>
       </c>
       <c r="F20" s="25">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G20" s="26"/>
       <c r="H20" s="12"/>
@@ -5117,22 +5114,20 @@
         <v>24</v>
       </c>
       <c r="B22" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46054</v>
       </c>
       <c r="C22" s="24">
-        <f>$B$4</f>
-        <v>46144</v>
+        <v>46070</v>
       </c>
       <c r="D22" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>16</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F22" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" s="26"/>
       <c r="H22" s="12"/>
@@ -5157,22 +5152,20 @@
         <v>25</v>
       </c>
       <c r="B23" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46057</v>
       </c>
       <c r="C23" s="24">
-        <f>$B$4</f>
-        <v>46144</v>
+        <v>46078</v>
       </c>
       <c r="D23" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>21</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F23" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="26"/>
       <c r="H23" s="12"/>
@@ -5197,22 +5190,20 @@
         <v>26</v>
       </c>
       <c r="B24" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46063</v>
       </c>
       <c r="C24" s="24">
-        <f>$B$4</f>
-        <v>46144</v>
+        <v>46096</v>
       </c>
       <c r="D24" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F24" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="26"/>
       <c r="H24" s="12"/>
@@ -5237,22 +5228,20 @@
         <v>29</v>
       </c>
       <c r="B25" s="24">
-        <f t="shared" ref="B25:B27" si="2">$B$3</f>
-        <v>46039</v>
+        <v>46064</v>
       </c>
       <c r="C25" s="24">
-        <f t="shared" ref="C25:C27" si="3">$B$4</f>
-        <v>46144</v>
+        <v>46122</v>
       </c>
       <c r="D25" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>58</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F25" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="26"/>
       <c r="H25" s="12"/>
@@ -5277,22 +5266,20 @@
         <v>30</v>
       </c>
       <c r="B26" s="24">
-        <f t="shared" si="2"/>
-        <v>46039</v>
+        <v>46063</v>
       </c>
       <c r="C26" s="24">
-        <f t="shared" si="3"/>
-        <v>46144</v>
+        <v>46114</v>
       </c>
       <c r="D26" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>51</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F26" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" s="26"/>
       <c r="H26" s="12"/>
@@ -5317,22 +5304,20 @@
         <v>31</v>
       </c>
       <c r="B27" s="24">
-        <f t="shared" si="2"/>
-        <v>46039</v>
+        <v>46091</v>
       </c>
       <c r="C27" s="24">
-        <f t="shared" si="3"/>
-        <v>46144</v>
+        <v>46122</v>
       </c>
       <c r="D27" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>31</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F27" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" s="26"/>
       <c r="H27" s="12"/>
@@ -5357,22 +5342,21 @@
         <v>28</v>
       </c>
       <c r="B28" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46082</v>
       </c>
       <c r="C28" s="24">
-        <f>$B$4</f>
-        <v>46144</v>
+        <f ca="1">B5</f>
+        <v>46143</v>
       </c>
       <c r="D28" s="23">
-        <f t="shared" si="1"/>
-        <v>105</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>61</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F28" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" s="26"/>
       <c r="H28" s="12"/>
@@ -7305,22 +7289,21 @@
         <v>32</v>
       </c>
       <c r="B30" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46127</v>
       </c>
       <c r="C30" s="24">
         <f>$B$4</f>
-        <v>46144</v>
+        <v>46143</v>
       </c>
       <c r="D30" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>16</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F30" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" s="26"/>
       <c r="H30" s="12"/>
@@ -7345,22 +7328,21 @@
         <v>33</v>
       </c>
       <c r="B31" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46129</v>
       </c>
       <c r="C31" s="24">
-        <f t="shared" ref="C31:C34" si="4">$B$4</f>
-        <v>46144</v>
+        <f t="shared" ref="C31:C34" si="2">$B$4</f>
+        <v>46143</v>
       </c>
       <c r="D31" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F31" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" s="26"/>
       <c r="H31" s="12"/>
@@ -7385,22 +7367,21 @@
         <v>34</v>
       </c>
       <c r="B32" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46124</v>
       </c>
       <c r="C32" s="24">
-        <f t="shared" si="4"/>
-        <v>46144</v>
+        <f t="shared" si="2"/>
+        <v>46143</v>
       </c>
       <c r="D32" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>19</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F32" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="26"/>
       <c r="H32" s="12"/>
@@ -7425,22 +7406,21 @@
         <v>35</v>
       </c>
       <c r="B33" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46132</v>
       </c>
       <c r="C33" s="24">
-        <f t="shared" si="4"/>
-        <v>46144</v>
+        <f t="shared" si="2"/>
+        <v>46143</v>
       </c>
       <c r="D33" s="23">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F33" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" s="26"/>
       <c r="H33" s="12"/>
@@ -7465,22 +7445,21 @@
         <v>36</v>
       </c>
       <c r="B34" s="24">
-        <f>$B$3</f>
-        <v>46039</v>
+        <v>46134</v>
       </c>
       <c r="C34" s="24">
-        <f t="shared" si="4"/>
-        <v>46144</v>
+        <f t="shared" si="2"/>
+        <v>46143</v>
       </c>
       <c r="D34" s="31">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>9</v>
       </c>
       <c r="E34" s="31" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F34" s="25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" s="26"/>
       <c r="H34" s="12"/>

</xml_diff>